<commit_message>
chore: remove unused file
</commit_message>
<xml_diff>
--- a/testdata/data_test_signup.xlsx
+++ b/testdata/data_test_signup.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Linh\Đồ án\Test-DA\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1085CDC9-20FB-4D2C-B4E1-065E4DF8B88D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70B118DB-9A07-4511-9EAD-2F869F638A2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{041962BD-50A0-4384-82B2-0A63E4228D89}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="44">
   <si>
     <t>first_name</t>
   </si>
@@ -162,6 +162,12 @@
   </si>
   <si>
     <t>aaaaaaaa</t>
+  </si>
+  <si>
+    <t>12Ngoclinh</t>
+  </si>
+  <si>
+    <t>Ngoclinh@</t>
   </si>
 </sst>
 </file>
@@ -574,7 +580,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BCA95D5-71D9-4607-8A55-30796E7D772D}">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17.83203125" style="3" customWidth="1"/>
@@ -1208,6 +1214,46 @@
         <v>424242</v>
       </c>
       <c r="F35" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E36" s="5">
+        <v>424242</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E37" s="5">
+        <v>424242</v>
+      </c>
+      <c r="F37" s="3" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1262,6 +1308,7 @@
     <hyperlink ref="C30:C31" r:id="rId47" display="ngoclinh+clerk_test@linky.now" xr:uid="{E89AF493-5A53-45AD-B8AF-4060403B6FA8}"/>
     <hyperlink ref="C32:C33" r:id="rId48" display="ngoclinh+clerk_test@linky.now" xr:uid="{B1156F0D-5073-4D37-B505-03E3589C0ED7}"/>
     <hyperlink ref="C28" r:id="rId49" xr:uid="{A65F5390-0866-4620-BC8E-976F1DBB4320}"/>
+    <hyperlink ref="D37" r:id="rId50" xr:uid="{E40FB1C4-7056-412B-9B4E-71F28BC68F8E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>